<commit_message>
task130 v3 repair 1: leak gate (implementation plan distractor, no evaluation-only line), pins (birth-month claims, CARC 18 duplicates, PBM processing window), realism (clinical coherence, catalogues, calendar, adjudication, containers, signatures); golden programme baseline $3,916 PMPM (medical $2,227, pharmacy $1,689); checks 5,972 pass, verifier green, rebuilds byte-identical, leak.py no LEAK
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01A6XcFx5t62c7gPi1bBKcVi
</commit_message>
<xml_diff>
--- a/task130/golden/cohort_baseline_2027.xlsx
+++ b/task130/golden/cohort_baseline_2027.xlsx
@@ -16,6 +16,143 @@
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
+</file>
+
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="44">
+  <si>
+    <t>Red Cedar Valley Schools Employee Health Plan</t>
+  </si>
+  <si>
+    <t>Northcourt care management: baseline for the Programme Year, 1 April 2027 to 31 March 2028</t>
+  </si>
+  <si>
+    <t>Certification under Schedule C.2 of Agreement RCV-2027-014. Prepared 12 March 2027 for the Board meeting of 25 March 2027.</t>
+  </si>
+  <si>
+    <t>Risk tier</t>
+  </si>
+  <si>
+    <t>Enrolled members</t>
+  </si>
+  <si>
+    <t>2026 allowed PMPM, medical</t>
+  </si>
+  <si>
+    <t>2026 allowed PMPM, pharmacy</t>
+  </si>
+  <si>
+    <t>Baseline PMPM, medical</t>
+  </si>
+  <si>
+    <t>Baseline PMPM, pharmacy</t>
+  </si>
+  <si>
+    <t>Tier 1</t>
+  </si>
+  <si>
+    <t>Tier 2</t>
+  </si>
+  <si>
+    <t>Tier 3</t>
+  </si>
+  <si>
+    <t>Tier 4</t>
+  </si>
+  <si>
+    <t>Programme baseline PMPM, tiers weighted by enrolled members</t>
+  </si>
+  <si>
+    <t>Medical</t>
+  </si>
+  <si>
+    <t>Pharmacy</t>
+  </si>
+  <si>
+    <t>Total</t>
+  </si>
+  <si>
+    <t>All enrolled members</t>
+  </si>
+  <si>
+    <t>Note 1. Whole dollars per member per month. No figure is rounded before the final figure (Schedule C.2), so a tier's medical and pharmacy figures are not added here.</t>
+  </si>
+  <si>
+    <t>Note 2. 2026 allowed PMPM: the enrolled members' allowed claims incurred in calendar 2026 and paid through 28 February 2027, not completed, over their 2026 member months (Schedule C.2).</t>
+  </si>
+  <si>
+    <t>Note 3. Baseline PMPM: allowed claims per member month, 1 April 2025 to 31 March 2026, of the members Northcourt's model placed in each tier on 2024 claims in its RFP 2025-07 proposal (never enrolled: the award was suspended in April 2025), counted for the months each was enrolled, and projected 24 months at the renewal trend, 6.5% medical and 9.0% pharmacy (Schedule C.1(g)).</t>
+  </si>
+  <si>
+    <t>Note 4. Allowed claims include member cost sharing, are net of replacement and void claims and pharmacy reversals, before manufacturer rebates and stop-loss reimbursements (Schedule C.1(a)). Member month: enrolled on the first of the month (Schedule C.1(b)).</t>
+  </si>
+  <si>
+    <t>Note 5. Sources: Ellery claim lines and eligibility, Quarrystone claims (pulled 1 to 3 March 2027); Ellery conversion file of 1 January 2025; Northcourt Final Enrolment List of 5 March 2027 and RFP 2025-07 stratification of 21 February 2025.</t>
+  </si>
+  <si>
+    <t>Members Northcourt placed in each tier on 2024 claims (RFP 2025-07, 21 February 2025), April 2025 to March 2026</t>
+  </si>
+  <si>
+    <t>Bramwell member numbers linked to Ellery member IDs through the conversion file; claims and months from 1 April 2025 to 31 March 2026.</t>
+  </si>
+  <si>
+    <t>Members on bid list</t>
+  </si>
+  <si>
+    <t>Enrolled on 1 April 2025</t>
+  </si>
+  <si>
+    <t>Member months</t>
+  </si>
+  <si>
+    <t>Medical allowed</t>
+  </si>
+  <si>
+    <t>Pharmacy allowed</t>
+  </si>
+  <si>
+    <t>Medical PMPM</t>
+  </si>
+  <si>
+    <t>Pharmacy PMPM</t>
+  </si>
+  <si>
+    <t>Trend factor, medical</t>
+  </si>
+  <si>
+    <t>Trend factor, pharmacy</t>
+  </si>
+  <si>
+    <t>All tiers</t>
+  </si>
+  <si>
+    <t>Trend: 1.065 and 1.09 a year (renewal letter of 26 February 2027) over the 24 months from the middle of the bid members' year (1 October 2025) to the middle of the Programme Year (1 October 2027).</t>
+  </si>
+  <si>
+    <t>Members who left the plan before 1 April 2025 have no member months in the year and drop out; members who left during it count for the months they were enrolled.</t>
+  </si>
+  <si>
+    <t>Members on Northcourt's Final Enrolment List (5 March 2027), calendar 2026, paid through 28 February 2027</t>
+  </si>
+  <si>
+    <t>2026 member months</t>
+  </si>
+  <si>
+    <t>Own 2026 PMPM at trend, medical</t>
+  </si>
+  <si>
+    <t>Own 2026 PMPM at trend, pharmacy</t>
+  </si>
+  <si>
+    <t>Columns H and I are for reference only and are not certified: each tier's own 2026 PMPM carried 15 months at trend, 1 July 2026 to 1 October 2027. Weighted by enrolled members they come to $7,205 medical and $1,690 pharmacy, $8,895 in total.</t>
+  </si>
+  <si>
+    <t>Northcourt chose these members because of their 2026 claims, so their 2026 level is not what they would be expected to cost in the Programme Year; see the Baseline sheet, note 3.</t>
+  </si>
+  <si>
+    <t>Where a member's coverage began partway through a month, as a newborn's does, that month's claims are included and the month is not a member month (Schedule C.1(a) and (b)).</t>
+  </si>
+</sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
@@ -548,181 +685,143 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Red Cedar Valley Schools Employee Health Plan</t>
-        </is>
+      <c r="A1" s="1" t="s">
+        <v>0</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Northcourt care management: baseline for the Programme Year, 1 April 2027 to 31 March 2028</t>
-        </is>
+      <c r="A2" s="2" t="s">
+        <v>1</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="3" t="inlineStr">
-        <is>
-          <t>Certification under Schedule C.2 of Agreement RCV-2027-014. Prepared 12 March 2027 for the Board meeting of 25 March 2027.</t>
-        </is>
+      <c r="A3" s="3" t="s">
+        <v>2</v>
       </c>
     </row>
     <row r="5" ht="46" customHeight="1">
-      <c r="A5" s="4" t="inlineStr">
-        <is>
-          <t>Risk tier</t>
-        </is>
-      </c>
-      <c r="B5" s="4" t="inlineStr">
-        <is>
-          <t>Enrolled members</t>
-        </is>
-      </c>
-      <c r="C5" s="4" t="inlineStr">
-        <is>
-          <t>2026 allowed PMPM, medical</t>
-        </is>
-      </c>
-      <c r="D5" s="4" t="inlineStr">
-        <is>
-          <t>2026 allowed PMPM, pharmacy</t>
-        </is>
-      </c>
-      <c r="E5" s="4" t="inlineStr">
-        <is>
-          <t>Baseline PMPM, medical</t>
-        </is>
-      </c>
-      <c r="F5" s="4" t="inlineStr">
-        <is>
-          <t>Baseline PMPM, pharmacy</t>
-        </is>
+      <c r="A5" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="D5" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="E5" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="F5" s="4" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="5" t="inlineStr">
-        <is>
-          <t>Tier 1</t>
-        </is>
+      <c r="A6" s="5" t="s">
+        <v>9</v>
       </c>
       <c r="B6" s="6" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="C6" s="7" t="n">
-        <v>15338</v>
+        <v>13317</v>
       </c>
       <c r="D6" s="7" t="n">
-        <v>2780</v>
+        <v>294</v>
       </c>
       <c r="E6" s="7" t="n">
-        <v>4177</v>
+        <v>5529</v>
       </c>
       <c r="F6" s="7" t="n">
-        <v>899</v>
+        <v>934</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="5" t="inlineStr">
-        <is>
-          <t>Tier 2</t>
-        </is>
+      <c r="A7" s="5" t="s">
+        <v>10</v>
       </c>
       <c r="B7" s="6" t="n">
+        <v>34</v>
+      </c>
+      <c r="C7" s="7" t="n">
+        <v>8914</v>
+      </c>
+      <c r="D7" s="7" t="n">
+        <v>1051</v>
+      </c>
+      <c r="E7" s="7" t="n">
+        <v>2660</v>
+      </c>
+      <c r="F7" s="7" t="n">
+        <v>2622</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="B8" s="6" t="n">
+        <v>48</v>
+      </c>
+      <c r="C8" s="7" t="n">
+        <v>4815</v>
+      </c>
+      <c r="D8" s="7" t="n">
+        <v>2056</v>
+      </c>
+      <c r="E8" s="7" t="n">
+        <v>1630</v>
+      </c>
+      <c r="F8" s="7" t="n">
+        <v>2241</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="B9" s="9" t="n">
         <v>38</v>
       </c>
-      <c r="C7" s="7" t="n">
-        <v>8182</v>
-      </c>
-      <c r="D7" s="7" t="n">
-        <v>1242</v>
-      </c>
-      <c r="E7" s="7" t="n">
-        <v>2729</v>
-      </c>
-      <c r="F7" s="7" t="n">
-        <v>2072</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="5" t="inlineStr">
-        <is>
-          <t>Tier 3</t>
-        </is>
-      </c>
-      <c r="B8" s="6" t="n">
-        <v>41</v>
-      </c>
-      <c r="C8" s="7" t="n">
-        <v>4828</v>
-      </c>
-      <c r="D8" s="7" t="n">
-        <v>1603</v>
-      </c>
-      <c r="E8" s="7" t="n">
-        <v>1172</v>
-      </c>
-      <c r="F8" s="7" t="n">
-        <v>1484</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="8" t="inlineStr">
-        <is>
-          <t>Tier 4</t>
-        </is>
-      </c>
-      <c r="B9" s="9" t="n">
-        <v>43</v>
-      </c>
       <c r="C9" s="10" t="n">
-        <v>3413</v>
+        <v>3468</v>
       </c>
       <c r="D9" s="10" t="n">
-        <v>1262</v>
+        <v>1899</v>
       </c>
       <c r="E9" s="10" t="n">
-        <v>1745</v>
+        <v>857</v>
       </c>
       <c r="F9" s="10" t="n">
-        <v>884</v>
+        <v>555</v>
       </c>
       <c r="G9" s="11" t="n"/>
     </row>
     <row r="11" ht="32" customHeight="1">
-      <c r="A11" s="12" t="inlineStr">
-        <is>
-          <t>Programme baseline PMPM, tiers weighted by enrolled members</t>
-        </is>
-      </c>
-      <c r="B11" s="4" t="inlineStr">
-        <is>
-          <t>Enrolled members</t>
-        </is>
+      <c r="A11" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="B11" s="4" t="s">
+        <v>4</v>
       </c>
       <c r="C11" s="4" t="n"/>
       <c r="D11" s="4" t="n"/>
-      <c r="E11" s="4" t="inlineStr">
-        <is>
-          <t>Medical</t>
-        </is>
-      </c>
-      <c r="F11" s="4" t="inlineStr">
-        <is>
-          <t>Pharmacy</t>
-        </is>
-      </c>
-      <c r="G11" s="4" t="inlineStr">
-        <is>
-          <t>Total</t>
-        </is>
+      <c r="E11" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="F11" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="G11" s="4" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="13" t="inlineStr">
-        <is>
-          <t>All enrolled members</t>
-        </is>
+      <c r="A12" s="13" t="s">
+        <v>17</v>
       </c>
       <c r="B12" s="14" t="n">
         <v>140</v>
@@ -730,48 +829,38 @@
       <c r="C12" s="15" t="n"/>
       <c r="D12" s="15" t="n"/>
       <c r="E12" s="15" t="n">
-        <v>2157</v>
+        <v>2227</v>
       </c>
       <c r="F12" s="15" t="n">
-        <v>1384</v>
+        <v>1689</v>
       </c>
       <c r="G12" s="15" t="n">
-        <v>3541</v>
+        <v>3916</v>
       </c>
     </row>
     <row r="14" ht="26" customHeight="1">
-      <c r="A14" s="16" t="inlineStr">
-        <is>
-          <t>Note 1. Whole dollars per member per month. No figure is rounded before the final figure (Schedule C.2), so a tier's medical and pharmacy figures are not added here.</t>
-        </is>
+      <c r="A14" s="16" t="s">
+        <v>18</v>
       </c>
     </row>
     <row r="15" ht="38" customHeight="1">
-      <c r="A15" s="16" t="inlineStr">
-        <is>
-          <t>Note 2. 2026 allowed PMPM: the enrolled members' allowed claims incurred in calendar 2026 and paid through 28 February 2027, not completed, over their 2026 member months (Schedule C.2).</t>
-        </is>
+      <c r="A15" s="16" t="s">
+        <v>19</v>
       </c>
     </row>
     <row r="16" ht="38" customHeight="1">
-      <c r="A16" s="16" t="inlineStr">
-        <is>
-          <t>Note 3. Baseline PMPM: allowed claims per member month, 1 April 2025 to 31 March 2026, of the members Northcourt's model placed in each tier on 2024 claims in its RFP 2025-07 proposal (never enrolled: the award was suspended in April 2025), counted for the months each was enrolled, and projected 24 months at the renewal trend, 6.5% medical and 9.0% pharmacy (Schedule C.1(g)).</t>
-        </is>
+      <c r="A16" s="16" t="s">
+        <v>20</v>
       </c>
     </row>
     <row r="17" ht="38" customHeight="1">
-      <c r="A17" s="16" t="inlineStr">
-        <is>
-          <t>Note 4. Allowed claims include member cost sharing, are net of replacement and void claims and pharmacy reversals, before manufacturer rebates and stop-loss reimbursements (Schedule C.1(a)). Member month: enrolled on the first of the month (Schedule C.1(b)).</t>
-        </is>
+      <c r="A17" s="16" t="s">
+        <v>21</v>
       </c>
     </row>
     <row r="18" ht="38" customHeight="1">
-      <c r="A18" s="16" t="inlineStr">
-        <is>
-          <t>Note 5. Sources: Ellery claim lines and eligibility, Quarrystone claims (pulled 1 to 3 March 2027); Ellery conversion file of 1 January 2025; Northcourt Final Enrolment List of 5 March 2027 and RFP 2025-07 stratification of 21 February 2025.</t>
-        </is>
+      <c r="A18" s="16" t="s">
+        <v>22</v>
       </c>
     </row>
   </sheetData>
@@ -811,107 +900,77 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="17" t="inlineStr">
-        <is>
-          <t>Members Northcourt placed in each tier on 2024 claims (RFP 2025-07, 21 February 2025), April 2025 to March 2026</t>
-        </is>
+      <c r="A1" s="17" t="s">
+        <v>23</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="18" t="inlineStr">
-        <is>
-          <t>Bramwell member numbers linked to Ellery member IDs through the conversion file; claims and months from 1 April 2025 to 31 March 2026.</t>
-        </is>
+      <c r="A2" s="18" t="s">
+        <v>24</v>
       </c>
     </row>
     <row r="4" ht="45" customHeight="1">
-      <c r="A4" s="19" t="inlineStr">
-        <is>
-          <t>Risk tier</t>
-        </is>
-      </c>
-      <c r="B4" s="19" t="inlineStr">
-        <is>
-          <t>Members on bid list</t>
-        </is>
-      </c>
-      <c r="C4" s="19" t="inlineStr">
-        <is>
-          <t>Enrolled on 1 April 2025</t>
-        </is>
-      </c>
-      <c r="D4" s="19" t="inlineStr">
-        <is>
-          <t>Member months</t>
-        </is>
-      </c>
-      <c r="E4" s="19" t="inlineStr">
-        <is>
-          <t>Medical allowed</t>
-        </is>
-      </c>
-      <c r="F4" s="19" t="inlineStr">
-        <is>
-          <t>Pharmacy allowed</t>
-        </is>
-      </c>
-      <c r="G4" s="19" t="inlineStr">
-        <is>
-          <t>Medical PMPM</t>
-        </is>
-      </c>
-      <c r="H4" s="19" t="inlineStr">
-        <is>
-          <t>Pharmacy PMPM</t>
-        </is>
-      </c>
-      <c r="I4" s="19" t="inlineStr">
-        <is>
-          <t>Trend factor, medical</t>
-        </is>
-      </c>
-      <c r="J4" s="19" t="inlineStr">
-        <is>
-          <t>Trend factor, pharmacy</t>
-        </is>
-      </c>
-      <c r="K4" s="19" t="inlineStr">
-        <is>
-          <t>Baseline PMPM, medical</t>
-        </is>
-      </c>
-      <c r="L4" s="19" t="inlineStr">
-        <is>
-          <t>Baseline PMPM, pharmacy</t>
-        </is>
+      <c r="A4" s="19" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" s="19" t="s">
+        <v>25</v>
+      </c>
+      <c r="C4" s="19" t="s">
+        <v>26</v>
+      </c>
+      <c r="D4" s="19" t="s">
+        <v>27</v>
+      </c>
+      <c r="E4" s="19" t="s">
+        <v>28</v>
+      </c>
+      <c r="F4" s="19" t="s">
+        <v>29</v>
+      </c>
+      <c r="G4" s="19" t="s">
+        <v>30</v>
+      </c>
+      <c r="H4" s="19" t="s">
+        <v>31</v>
+      </c>
+      <c r="I4" s="19" t="s">
+        <v>32</v>
+      </c>
+      <c r="J4" s="19" t="s">
+        <v>33</v>
+      </c>
+      <c r="K4" s="19" t="s">
+        <v>7</v>
+      </c>
+      <c r="L4" s="19" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Tier 1</t>
-        </is>
+      <c r="A5" t="s">
+        <v>9</v>
       </c>
       <c r="B5" s="20" t="n">
+        <v>18</v>
+      </c>
+      <c r="C5" s="20" t="n">
         <v>17</v>
       </c>
-      <c r="C5" s="20" t="n">
-        <v>14</v>
-      </c>
       <c r="D5" s="20" t="n">
-        <v>147</v>
+        <v>172</v>
       </c>
       <c r="E5" s="21" t="n">
-        <v>541389.25</v>
+        <v>838468.63</v>
       </c>
       <c r="F5" s="21" t="n">
-        <v>111247.86</v>
+        <v>135193.94</v>
       </c>
       <c r="G5" s="21" t="n">
-        <v>3682.92</v>
+        <v>4874.82</v>
       </c>
       <c r="H5" s="21" t="n">
-        <v>756.79</v>
+        <v>786.01</v>
       </c>
       <c r="I5" s="22" t="n">
         <v>1.134225</v>
@@ -920,38 +979,36 @@
         <v>1.1881</v>
       </c>
       <c r="K5" s="21" t="n">
-        <v>4177.26</v>
+        <v>5529.14</v>
       </c>
       <c r="L5" s="21" t="n">
-        <v>899.14</v>
+        <v>933.86</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Tier 2</t>
-        </is>
+      <c r="A6" t="s">
+        <v>10</v>
       </c>
       <c r="B6" s="20" t="n">
-        <v>41</v>
+        <v>31</v>
       </c>
       <c r="C6" s="20" t="n">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="D6" s="20" t="n">
-        <v>441</v>
+        <v>344</v>
       </c>
       <c r="E6" s="21" t="n">
-        <v>1061121.68</v>
+        <v>806711.05</v>
       </c>
       <c r="F6" s="21" t="n">
-        <v>769034.8100000001</v>
+        <v>759104.72</v>
       </c>
       <c r="G6" s="21" t="n">
-        <v>2406.17</v>
+        <v>2345.09</v>
       </c>
       <c r="H6" s="21" t="n">
-        <v>1743.84</v>
+        <v>2206.7</v>
       </c>
       <c r="I6" s="22" t="n">
         <v>1.134225</v>
@@ -960,38 +1017,36 @@
         <v>1.1881</v>
       </c>
       <c r="K6" s="21" t="n">
-        <v>2729.14</v>
+        <v>2659.86</v>
       </c>
       <c r="L6" s="21" t="n">
-        <v>2071.86</v>
+        <v>2621.78</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Tier 3</t>
-        </is>
+      <c r="A7" t="s">
+        <v>11</v>
       </c>
       <c r="B7" s="20" t="n">
-        <v>27</v>
+        <v>47</v>
       </c>
       <c r="C7" s="20" t="n">
-        <v>26</v>
+        <v>45</v>
       </c>
       <c r="D7" s="20" t="n">
-        <v>312</v>
+        <v>526</v>
       </c>
       <c r="E7" s="21" t="n">
-        <v>322451.58</v>
+        <v>755777.91</v>
       </c>
       <c r="F7" s="21" t="n">
-        <v>389667.81</v>
+        <v>992081.78</v>
       </c>
       <c r="G7" s="21" t="n">
-        <v>1033.5</v>
+        <v>1436.84</v>
       </c>
       <c r="H7" s="21" t="n">
-        <v>1248.94</v>
+        <v>1886.09</v>
       </c>
       <c r="I7" s="22" t="n">
         <v>1.134225</v>
@@ -1000,38 +1055,36 @@
         <v>1.1881</v>
       </c>
       <c r="K7" s="21" t="n">
-        <v>1172.22</v>
+        <v>1629.7</v>
       </c>
       <c r="L7" s="21" t="n">
-        <v>1483.86</v>
+        <v>2240.86</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Tier 4</t>
-        </is>
+      <c r="A8" t="s">
+        <v>12</v>
       </c>
       <c r="B8" s="20" t="n">
-        <v>55</v>
+        <v>44</v>
       </c>
       <c r="C8" s="20" t="n">
-        <v>53</v>
+        <v>44</v>
       </c>
       <c r="D8" s="20" t="n">
-        <v>566</v>
+        <v>500</v>
       </c>
       <c r="E8" s="21" t="n">
-        <v>870898.21</v>
+        <v>377694.02</v>
       </c>
       <c r="F8" s="21" t="n">
-        <v>421272.45</v>
+        <v>233692.45</v>
       </c>
       <c r="G8" s="21" t="n">
-        <v>1538.69</v>
+        <v>755.39</v>
       </c>
       <c r="H8" s="21" t="n">
-        <v>744.3</v>
+        <v>467.38</v>
       </c>
       <c r="I8" s="22" t="n">
         <v>1.134225</v>
@@ -1040,46 +1093,40 @@
         <v>1.1881</v>
       </c>
       <c r="K8" s="21" t="n">
-        <v>1745.22</v>
+        <v>856.78</v>
       </c>
       <c r="L8" s="21" t="n">
-        <v>884.3</v>
+        <v>555.3</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="23" t="inlineStr">
-        <is>
-          <t>All tiers</t>
-        </is>
+      <c r="A9" s="23" t="s">
+        <v>34</v>
       </c>
       <c r="B9" s="24" t="n">
         <v>140</v>
       </c>
       <c r="C9" s="24" t="n">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="D9" s="24" t="n">
-        <v>1466</v>
+        <v>1542</v>
       </c>
       <c r="E9" s="25" t="n">
-        <v>2795860.72</v>
+        <v>2778651.61</v>
       </c>
       <c r="F9" s="25" t="n">
-        <v>1691222.93</v>
+        <v>2120072.89</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="26" t="inlineStr">
-        <is>
-          <t>Trend: 1.065 and 1.09 a year (renewal letter of 26 February 2027) over the 24 months from the middle of the bid members' year (1 October 2025) to the middle of the Programme Year (1 October 2027).</t>
-        </is>
+      <c r="A11" s="26" t="s">
+        <v>35</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="26" t="inlineStr">
-        <is>
-          <t>Members who left the plan before 1 April 2025 have no member months in the year and drop out; members who left during it count for the months they were enrolled.</t>
-        </is>
+      <c r="A12" s="26" t="s">
+        <v>36</v>
       </c>
     </row>
   </sheetData>
@@ -1094,7 +1141,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I10"/>
+  <dimension ref="A1:I11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1109,195 +1156,168 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="17" t="inlineStr">
-        <is>
-          <t>Members on Northcourt's Final Enrolment List (5 March 2027), calendar 2026, paid through 28 February 2027</t>
-        </is>
+      <c r="A1" s="17" t="s">
+        <v>37</v>
       </c>
     </row>
     <row r="3" ht="45" customHeight="1">
-      <c r="A3" s="19" t="inlineStr">
-        <is>
-          <t>Risk tier</t>
-        </is>
-      </c>
-      <c r="B3" s="19" t="inlineStr">
-        <is>
-          <t>Enrolled members</t>
-        </is>
-      </c>
-      <c r="C3" s="19" t="inlineStr">
-        <is>
-          <t>2026 member months</t>
-        </is>
-      </c>
-      <c r="D3" s="19" t="inlineStr">
-        <is>
-          <t>Medical allowed</t>
-        </is>
-      </c>
-      <c r="E3" s="19" t="inlineStr">
-        <is>
-          <t>Pharmacy allowed</t>
-        </is>
-      </c>
-      <c r="F3" s="19" t="inlineStr">
-        <is>
-          <t>Medical PMPM</t>
-        </is>
-      </c>
-      <c r="G3" s="19" t="inlineStr">
-        <is>
-          <t>Pharmacy PMPM</t>
-        </is>
-      </c>
-      <c r="H3" s="19" t="inlineStr">
-        <is>
-          <t>Own 2026 PMPM at trend, medical</t>
-        </is>
-      </c>
-      <c r="I3" s="19" t="inlineStr">
-        <is>
-          <t>Own 2026 PMPM at trend, pharmacy</t>
-        </is>
+      <c r="A3" s="19" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" s="19" t="s">
+        <v>4</v>
+      </c>
+      <c r="C3" s="19" t="s">
+        <v>38</v>
+      </c>
+      <c r="D3" s="19" t="s">
+        <v>28</v>
+      </c>
+      <c r="E3" s="19" t="s">
+        <v>29</v>
+      </c>
+      <c r="F3" s="19" t="s">
+        <v>30</v>
+      </c>
+      <c r="G3" s="19" t="s">
+        <v>31</v>
+      </c>
+      <c r="H3" s="19" t="s">
+        <v>39</v>
+      </c>
+      <c r="I3" s="19" t="s">
+        <v>40</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Tier 1</t>
-        </is>
+      <c r="A4" t="s">
+        <v>9</v>
       </c>
       <c r="B4" s="20" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="C4" s="20" t="n">
-        <v>205</v>
+        <v>233</v>
       </c>
       <c r="D4" s="21" t="n">
-        <v>3144341.25</v>
+        <v>3102797.56</v>
       </c>
       <c r="E4" s="21" t="n">
-        <v>569951.25</v>
+        <v>68545.32000000001</v>
       </c>
       <c r="F4" s="21" t="n">
-        <v>15338.25</v>
+        <v>13316.73</v>
       </c>
       <c r="G4" s="21" t="n">
-        <v>2780.25</v>
+        <v>294.19</v>
       </c>
       <c r="H4" s="21" t="n">
-        <v>16594.45</v>
+        <v>14407.36</v>
       </c>
       <c r="I4" s="21" t="n">
-        <v>3096.47</v>
+        <v>327.65</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Tier 2</t>
-        </is>
+      <c r="A5" t="s">
+        <v>10</v>
       </c>
       <c r="B5" s="20" t="n">
+        <v>34</v>
+      </c>
+      <c r="C5" s="20" t="n">
+        <v>395</v>
+      </c>
+      <c r="D5" s="21" t="n">
+        <v>3520956.23</v>
+      </c>
+      <c r="E5" s="21" t="n">
+        <v>415243.75</v>
+      </c>
+      <c r="F5" s="21" t="n">
+        <v>8913.809999999999</v>
+      </c>
+      <c r="G5" s="21" t="n">
+        <v>1051.25</v>
+      </c>
+      <c r="H5" s="21" t="n">
+        <v>9643.85</v>
+      </c>
+      <c r="I5" s="21" t="n">
+        <v>1170.82</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="s">
+        <v>11</v>
+      </c>
+      <c r="B6" s="20" t="n">
+        <v>48</v>
+      </c>
+      <c r="C6" s="20" t="n">
+        <v>564</v>
+      </c>
+      <c r="D6" s="21" t="n">
+        <v>2715519</v>
+      </c>
+      <c r="E6" s="21" t="n">
+        <v>1159693.11</v>
+      </c>
+      <c r="F6" s="21" t="n">
+        <v>4814.75</v>
+      </c>
+      <c r="G6" s="21" t="n">
+        <v>2056.19</v>
+      </c>
+      <c r="H6" s="21" t="n">
+        <v>5209.08</v>
+      </c>
+      <c r="I6" s="21" t="n">
+        <v>2290.06</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="s">
+        <v>12</v>
+      </c>
+      <c r="B7" s="20" t="n">
         <v>38</v>
       </c>
-      <c r="C5" s="20" t="n">
-        <v>451</v>
-      </c>
-      <c r="D5" s="21" t="n">
-        <v>3689985.08</v>
-      </c>
-      <c r="E5" s="21" t="n">
-        <v>560273.58</v>
-      </c>
-      <c r="F5" s="21" t="n">
-        <v>8181.79</v>
-      </c>
-      <c r="G5" s="21" t="n">
-        <v>1242.29</v>
-      </c>
-      <c r="H5" s="21" t="n">
-        <v>8851.870000000001</v>
-      </c>
-      <c r="I5" s="21" t="n">
-        <v>1383.59</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Tier 3</t>
-        </is>
-      </c>
-      <c r="B6" s="20" t="n">
+      <c r="C7" s="20" t="n">
+        <v>442</v>
+      </c>
+      <c r="D7" s="21" t="n">
+        <v>1532738.08</v>
+      </c>
+      <c r="E7" s="21" t="n">
+        <v>839468.5</v>
+      </c>
+      <c r="F7" s="21" t="n">
+        <v>3467.73</v>
+      </c>
+      <c r="G7" s="21" t="n">
+        <v>1899.25</v>
+      </c>
+      <c r="H7" s="21" t="n">
+        <v>3751.74</v>
+      </c>
+      <c r="I7" s="21" t="n">
+        <v>2115.27</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="26" t="s">
         <v>41</v>
       </c>
-      <c r="C6" s="20" t="n">
-        <v>485</v>
-      </c>
-      <c r="D6" s="21" t="n">
-        <v>2341649.35</v>
-      </c>
-      <c r="E6" s="21" t="n">
-        <v>777576.25</v>
-      </c>
-      <c r="F6" s="21" t="n">
-        <v>4828.14</v>
-      </c>
-      <c r="G6" s="21" t="n">
-        <v>1603.25</v>
-      </c>
-      <c r="H6" s="21" t="n">
-        <v>5223.57</v>
-      </c>
-      <c r="I6" s="21" t="n">
-        <v>1785.6</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Tier 4</t>
-        </is>
-      </c>
-      <c r="B7" s="20" t="n">
+    </row>
+    <row r="10">
+      <c r="A10" s="26" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="26" t="s">
         <v>43</v>
-      </c>
-      <c r="C7" s="20" t="n">
-        <v>495</v>
-      </c>
-      <c r="D7" s="21" t="n">
-        <v>1689311.25</v>
-      </c>
-      <c r="E7" s="21" t="n">
-        <v>624566.25</v>
-      </c>
-      <c r="F7" s="21" t="n">
-        <v>3412.75</v>
-      </c>
-      <c r="G7" s="21" t="n">
-        <v>1261.75</v>
-      </c>
-      <c r="H7" s="21" t="n">
-        <v>3692.25</v>
-      </c>
-      <c r="I7" s="21" t="n">
-        <v>1405.26</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="26" t="inlineStr">
-        <is>
-          <t>Columns H and I are for reference only and are not certified: each tier's own 2026 PMPM carried 15 months at trend, 1 July 2026 to 1 October 2027. Weighted by enrolled members they come to $7,200 medical and $1,728 pharmacy, $8,928 in total.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="26" t="inlineStr">
-        <is>
-          <t>Northcourt chose these members because of their 2026 claims, so their 2026 level is not what they would be expected to cost in the Programme Year; see the Baseline sheet, note 3.</t>
-        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
task130 repair r4: centre every graded figure off round values; golden programme baseline unchanged at $4,060 PMPM (medical $1,438, pharmacy $2,622)
The tuner aimed the tier baselines at two-decimal values and the 2026 PMPMs at
quarter-dollars, so a full-precision figure came out exact only under the
intended method (a confirming bell). tune.py now draws each figure's offset in
its bin from a seeded generator (seed 52389), builds and measures every draw,
and keeps one only when every rung's and fork's programme total is off the
cent grid too. checks.py asserts the 0.0005 floors off the cent and
quarter-dollar grids for all 19 graded figures and every rung and fork total;
verify.py checks the graded figures independently. No whole-dollar figure
moved; the renewal letter's exhibits move by $0.01 to $38.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01A6XcFx5t62c7gPi1bBKcVi
</commit_message>
<xml_diff>
--- a/task130/golden/cohort_baseline_2027.xlsx
+++ b/task130/golden/cohort_baseline_2027.xlsx
@@ -961,16 +961,16 @@
         <v>440</v>
       </c>
       <c r="E5" s="21" t="n">
-        <v>1170501.44</v>
+        <v>1170499.35</v>
       </c>
       <c r="F5" s="21" t="n">
-        <v>1196469.66</v>
+        <v>1196478.46</v>
       </c>
       <c r="G5" s="21" t="n">
         <v>2660.23</v>
       </c>
       <c r="H5" s="21" t="n">
-        <v>2719.25</v>
+        <v>2719.27</v>
       </c>
       <c r="I5" s="22" t="n">
         <v>1.134225</v>
@@ -979,10 +979,10 @@
         <v>1.1881</v>
       </c>
       <c r="K5" s="21" t="n">
-        <v>3017.3</v>
+        <v>3017.29</v>
       </c>
       <c r="L5" s="21" t="n">
-        <v>3230.74</v>
+        <v>3230.76</v>
       </c>
     </row>
     <row r="6">
@@ -999,16 +999,16 @@
         <v>333</v>
       </c>
       <c r="E6" s="21" t="n">
-        <v>366174.49</v>
+        <v>366172.69</v>
       </c>
       <c r="F6" s="21" t="n">
-        <v>654491.73</v>
+        <v>654494.9</v>
       </c>
       <c r="G6" s="21" t="n">
         <v>1099.62</v>
       </c>
       <c r="H6" s="21" t="n">
-        <v>1965.44</v>
+        <v>1965.45</v>
       </c>
       <c r="I6" s="22" t="n">
         <v>1.134225</v>
@@ -1017,10 +1017,10 @@
         <v>1.1881</v>
       </c>
       <c r="K6" s="21" t="n">
-        <v>1247.22</v>
+        <v>1247.21</v>
       </c>
       <c r="L6" s="21" t="n">
-        <v>2335.14</v>
+        <v>2335.15</v>
       </c>
     </row>
     <row r="7">
@@ -1037,16 +1037,16 @@
         <v>253</v>
       </c>
       <c r="E7" s="21" t="n">
-        <v>146358.46</v>
+        <v>146359.8</v>
       </c>
       <c r="F7" s="21" t="n">
-        <v>590100.51</v>
+        <v>590101.12</v>
       </c>
       <c r="G7" s="21" t="n">
-        <v>578.49</v>
+        <v>578.5</v>
       </c>
       <c r="H7" s="21" t="n">
-        <v>2332.41</v>
+        <v>2332.42</v>
       </c>
       <c r="I7" s="22" t="n">
         <v>1.134225</v>
@@ -1055,7 +1055,7 @@
         <v>1.1881</v>
       </c>
       <c r="K7" s="21" t="n">
-        <v>656.14</v>
+        <v>656.15</v>
       </c>
       <c r="L7" s="21" t="n">
         <v>2771.14</v>
@@ -1075,16 +1075,16 @@
         <v>528</v>
       </c>
       <c r="E8" s="21" t="n">
-        <v>415826.91</v>
+        <v>415815.42</v>
       </c>
       <c r="F8" s="21" t="n">
-        <v>939165.39</v>
+        <v>939150.27</v>
       </c>
       <c r="G8" s="21" t="n">
-        <v>787.55</v>
+        <v>787.53</v>
       </c>
       <c r="H8" s="21" t="n">
-        <v>1778.72</v>
+        <v>1778.69</v>
       </c>
       <c r="I8" s="22" t="n">
         <v>1.134225</v>
@@ -1093,10 +1093,10 @@
         <v>1.1881</v>
       </c>
       <c r="K8" s="21" t="n">
-        <v>893.26</v>
+        <v>893.24</v>
       </c>
       <c r="L8" s="21" t="n">
-        <v>2113.3</v>
+        <v>2113.27</v>
       </c>
     </row>
     <row r="9">
@@ -1113,10 +1113,10 @@
         <v>1554</v>
       </c>
       <c r="E9" s="25" t="n">
-        <v>2098861.3</v>
+        <v>2098847.26</v>
       </c>
       <c r="F9" s="25" t="n">
-        <v>3380227.29</v>
+        <v>3380224.75</v>
       </c>
     </row>
     <row r="11">
@@ -1200,22 +1200,22 @@
         <v>389</v>
       </c>
       <c r="D4" s="21" t="n">
-        <v>3739519.32</v>
+        <v>3739518.58</v>
       </c>
       <c r="E4" s="21" t="n">
-        <v>1048841.25</v>
+        <v>1048858.78</v>
       </c>
       <c r="F4" s="21" t="n">
         <v>9613.16</v>
       </c>
       <c r="G4" s="21" t="n">
-        <v>2696.25</v>
+        <v>2696.3</v>
       </c>
       <c r="H4" s="21" t="n">
-        <v>10400.48</v>
+        <v>10400.47</v>
       </c>
       <c r="I4" s="21" t="n">
-        <v>3002.92</v>
+        <v>3002.97</v>
       </c>
     </row>
     <row r="5">
@@ -1229,22 +1229,22 @@
         <v>429</v>
       </c>
       <c r="D5" s="21" t="n">
-        <v>1859822.25</v>
+        <v>1859840.83</v>
       </c>
       <c r="E5" s="21" t="n">
-        <v>1390925.25</v>
+        <v>1390932.11</v>
       </c>
       <c r="F5" s="21" t="n">
-        <v>4335.25</v>
+        <v>4335.29</v>
       </c>
       <c r="G5" s="21" t="n">
-        <v>3242.25</v>
+        <v>3242.27</v>
       </c>
       <c r="H5" s="21" t="n">
-        <v>4690.31</v>
+        <v>4690.35</v>
       </c>
       <c r="I5" s="21" t="n">
-        <v>3611.02</v>
+        <v>3611.04</v>
       </c>
     </row>
     <row r="6">
@@ -1258,22 +1258,22 @@
         <v>433</v>
       </c>
       <c r="D6" s="21" t="n">
-        <v>1513226.75</v>
+        <v>1513221.06</v>
       </c>
       <c r="E6" s="21" t="n">
-        <v>1104691.25</v>
+        <v>1104640.58</v>
       </c>
       <c r="F6" s="21" t="n">
-        <v>3494.75</v>
+        <v>3494.74</v>
       </c>
       <c r="G6" s="21" t="n">
-        <v>2551.25</v>
+        <v>2551.13</v>
       </c>
       <c r="H6" s="21" t="n">
-        <v>3780.97</v>
+        <v>3780.95</v>
       </c>
       <c r="I6" s="21" t="n">
-        <v>2841.42</v>
+        <v>2841.29</v>
       </c>
     </row>
     <row r="7">
@@ -1287,22 +1287,22 @@
         <v>361</v>
       </c>
       <c r="D7" s="21" t="n">
-        <v>692849.25</v>
+        <v>692855.6</v>
       </c>
       <c r="E7" s="21" t="n">
-        <v>1644625.75</v>
+        <v>1644613.29</v>
       </c>
       <c r="F7" s="21" t="n">
-        <v>1919.25</v>
+        <v>1919.27</v>
       </c>
       <c r="G7" s="21" t="n">
-        <v>4555.75</v>
+        <v>4555.72</v>
       </c>
       <c r="H7" s="21" t="n">
-        <v>2076.44</v>
+        <v>2076.46</v>
       </c>
       <c r="I7" s="21" t="n">
-        <v>5073.91</v>
+        <v>5073.87</v>
       </c>
     </row>
     <row r="9">

</xml_diff>